<commit_message>
Updated files for revision
New analyses with leave-one-out cross-validation, correlation, and calibration parameters.
</commit_message>
<xml_diff>
--- a/Data/VisualSiteClassification.xlsx
+++ b/Data/VisualSiteClassification.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbecker14\Documents\CRNS_USGS_Analysis\VegIndicesAnalysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbecker14\Documents\GitHub\CRNS_in_Roaring_Fork_CO\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B2F5C8-C85E-4A63-A870-01C98789D2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC02EB0-63B0-43DD-B81F-A968B8CFE3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28875" yWindow="1845" windowWidth="13620" windowHeight="11175" xr2:uid="{CDB15264-A0E7-477A-B8DA-8729047A7CEB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CDB15264-A0E7-477A-B8DA-8729047A7CEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,7 @@
   <authors>
     <author>tc={5CD22071-551C-4B6B-8300-086F6E4C5026}</author>
     <author>tc={04ECD8C1-0E08-434F-A51B-5E3E87CEAAEF}</author>
+    <author>tc={480B3030-77AC-4BB2-A01F-9051F74F2DE9}</author>
   </authors>
   <commentList>
     <comment ref="D6" authorId="0" shapeId="0" xr:uid="{5CD22071-551C-4B6B-8300-086F6E4C5026}">
@@ -56,6 +57,16 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Updated 4/29/25</t>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="2" shapeId="0" xr:uid="{480B3030-77AC-4BB2-A01F-9051F74F2DE9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Updated 12/12/2025 because of shrubby oaks on outskirts, riparian trees
+Reply:
+    Changed back</t>
       </text>
     </comment>
   </commentList>
@@ -575,19 +586,25 @@
   <threadedComment ref="D8" dT="2025-04-29T18:18:46.42" personId="{7105DEE9-CCA4-4C07-8123-6B4FB057658D}" id="{04ECD8C1-0E08-434F-A51B-5E3E87CEAAEF}">
     <text>Updated 4/29/25</text>
   </threadedComment>
+  <threadedComment ref="D9" dT="2025-12-12T16:04:18.22" personId="{7105DEE9-CCA4-4C07-8123-6B4FB057658D}" id="{480B3030-77AC-4BB2-A01F-9051F74F2DE9}">
+    <text>Updated 12/12/2025 because of shrubby oaks on outskirts, riparian trees</text>
+  </threadedComment>
+  <threadedComment ref="D9" dT="2025-12-14T14:57:42.09" personId="{7105DEE9-CCA4-4C07-8123-6B4FB057658D}" id="{93B4627B-76EF-4E06-B775-47C81ADEE924}" parentId="{480B3030-77AC-4BB2-A01F-9051F74F2DE9}">
+    <text>Changed back</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A705745C-01BD-4761-901B-0002D443EFBB}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" customWidth="1"/>
-    <col min="3" max="3" width="38.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -601,7 +618,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -615,7 +632,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -629,7 +646,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -643,7 +660,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -657,7 +674,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -671,7 +688,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -685,7 +702,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -699,7 +716,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -713,7 +730,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -727,7 +744,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -741,7 +758,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -755,7 +772,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -769,7 +786,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -783,7 +800,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -797,7 +814,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -811,7 +828,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -819,7 +836,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -827,7 +844,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -835,7 +852,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -843,7 +860,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>35</v>
       </c>

</xml_diff>